<commit_message>
Commit 2, codigo sencillo
</commit_message>
<xml_diff>
--- a/config/parametros.xlsx
+++ b/config/parametros.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diana.acosta\Desktop\CURSO PYTHON\EJERCICIO 3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8E8E57-4708-4339-BF58-807FB198A41A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CB6EBD-BECE-433C-98E0-DDAC0C5185F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{879D70DC-1290-40BB-97D4-36867B0286A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{879D70DC-1290-40BB-97D4-36867B0286A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros" sheetId="1" r:id="rId1"/>
-    <sheet name="Cargos" sheetId="2" r:id="rId2"/>
-    <sheet name="Centros_Costos" sheetId="3" r:id="rId3"/>
-    <sheet name="Matriz_Roles" sheetId="4" r:id="rId4"/>
-    <sheet name="Campos_Obligatorios" sheetId="5" r:id="rId5"/>
+    <sheet name="cargos" sheetId="2" r:id="rId2"/>
+    <sheet name="centros_costo" sheetId="3" r:id="rId3"/>
+    <sheet name="matriz_roles" sheetId="4" r:id="rId4"/>
+    <sheet name="campos_requeridos" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,16 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="119">
-  <si>
-    <t>Valor</t>
-  </si>
-  <si>
-    <t>Descripcion</t>
-  </si>
-  <si>
-    <t>Clave</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="121">
   <si>
     <t>dominio_correo</t>
   </si>
@@ -321,21 +312,6 @@
     <t>requiere_aprobacion</t>
   </si>
   <si>
-    <t>PER_ANALISTA_BAS</t>
-  </si>
-  <si>
-    <t>PER_ANALISTA_AVZ</t>
-  </si>
-  <si>
-    <t>PER_DESARROLLO</t>
-  </si>
-  <si>
-    <t>PERF_CONSULTOR</t>
-  </si>
-  <si>
-    <t>PERF_ADMIN_BAS</t>
-  </si>
-  <si>
     <t>PERF_GERENCIAL</t>
   </si>
   <si>
@@ -345,30 +321,12 @@
     <t>SI</t>
   </si>
   <si>
-    <t>PERF_ANALISTA_DATOS</t>
-  </si>
-  <si>
-    <t>PERF_DESARROLLO_AVZ</t>
-  </si>
-  <si>
     <t>PERF_ASIST_ADMIN</t>
   </si>
   <si>
-    <t>PERF_SOPORTE</t>
-  </si>
-  <si>
     <t>PERF_ANALISTA_FIN</t>
   </si>
   <si>
-    <t>PERF_CONSULTOR_AVZ</t>
-  </si>
-  <si>
-    <t>PERF_GER_TECNOLOGIA</t>
-  </si>
-  <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>tipo_novedad</t>
   </si>
   <si>
@@ -400,6 +358,54 @@
   </si>
   <si>
     <t>Consultor Junior</t>
+  </si>
+  <si>
+    <t>clave</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>descripcion</t>
+  </si>
+  <si>
+    <t>PERF_ADMIN_ADM</t>
+  </si>
+  <si>
+    <t>PERF_ANALISTA_RH</t>
+  </si>
+  <si>
+    <t>PERF_ANL_SN</t>
+  </si>
+  <si>
+    <t>PERF_ANL_JN</t>
+  </si>
+  <si>
+    <t>PERF_SOPOR_AVZ</t>
+  </si>
+  <si>
+    <t>PER_ANALISTA_DAT</t>
+  </si>
+  <si>
+    <t>PER_CONSUL_FUN</t>
+  </si>
+  <si>
+    <t>PERF_CONS_JN</t>
+  </si>
+  <si>
+    <t>PER_CONS_SN</t>
+  </si>
+  <si>
+    <t>PERF_DESA_SMS</t>
+  </si>
+  <si>
+    <t>PERF_DESA_SENIOR</t>
+  </si>
+  <si>
+    <t>PERF_DESA_JN</t>
+  </si>
+  <si>
+    <t>PERF_GEREN_TI</t>
   </si>
 </sst>
 </file>
@@ -429,7 +435,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -437,16 +443,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom style="thin">
+        <color theme="7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,9 +861,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF8BE932-52D6-4FC7-B7C1-B33E2AFBE485}" name="Table1" displayName="Table1" ref="A1:C8" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:C8" xr:uid="{DF8BE932-52D6-4FC7-B7C1-B33E2AFBE485}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BEA7E694-A666-4EA3-9758-BB238C66DC17}" name="Clave" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{D8AE14C3-4E8B-47AD-B406-84B30769DAA3}" name="Valor" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{2C5C5407-EE87-463D-97F8-3C8148D5F844}" name="Descripcion" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{BEA7E694-A666-4EA3-9758-BB238C66DC17}" name="clave" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{D8AE14C3-4E8B-47AD-B406-84B30769DAA3}" name="valor" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{2C5C5407-EE87-463D-97F8-3C8148D5F844}" name="descripcion" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -873,27 +901,27 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}" name="Table4" displayName="Table4" ref="A1:D14" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:D14" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}" name="Table4" displayName="Table4" ref="A1:D17" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:D17" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D14">
     <sortCondition ref="B2:B14"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{473C91A2-BCF7-4D6F-8BF6-61E64B46CCE0}" name="codigo_cargo" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{69A88768-23BB-486C-A0F0-79610F1F7C44}" name="area" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{68BAB88F-0803-48CA-B1F8-E65F18641620}" name="perfil_sistema" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{A1528DB0-D591-4C7B-A8FB-319135B195EE}" name="requiere_aprobacion" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{473C91A2-BCF7-4D6F-8BF6-61E64B46CCE0}" name="codigo_cargo" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{69A88768-23BB-486C-A0F0-79610F1F7C44}" name="area" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{68BAB88F-0803-48CA-B1F8-E65F18641620}" name="perfil_sistema" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{A1528DB0-D591-4C7B-A8FB-319135B195EE}" name="requiere_aprobacion" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}" name="Table5" displayName="Table5" ref="A1:B5" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}" name="Table5" displayName="Table5" ref="A1:B5" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A1:B5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DFC6A082-5976-4820-A3F4-184DF08ECDEE}" name="tipo_novedad" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{3110F81E-BAA3-466D-B6AE-46186B9CD74D}" name="campos_requeridos" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{DFC6A082-5976-4820-A3F4-184DF08ECDEE}" name="tipo_novedad" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{3110F81E-BAA3-466D-B6AE-46186B9CD74D}" name="campos_requeridos" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1226,90 +1254,90 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>120</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2">
         <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1333,240 +1361,240 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C5" s="1">
         <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C9" s="1">
         <v>2</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C10" s="1">
         <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C11" s="1">
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="C12" s="1">
         <v>2</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C13" s="1">
         <v>2</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C14" s="1">
         <v>3</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C15" s="1">
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C16" s="1">
         <v>5</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C17" s="1">
         <v>5</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1590,167 +1618,167 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1763,213 +1791,269 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8187E3A6-A1A2-45FF-B332-60C475BF706B}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>98</v>
-      </c>
+      <c r="C16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1984,48 +2068,48 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="93.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2213,20 +2297,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="66a9638b-dd80-4936-9407-2514d3c973e6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="66a9638b-dd80-4936-9407-2514d3c973e6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2248,14 +2332,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44E69664-3D00-4936-861C-A6F515DC2017}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2AE3EE-F1E3-4335-849F-CA480FA8E060}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -2269,4 +2345,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44E69664-3D00-4936-861C-A6F515DC2017}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revision y correccion de los errores
</commit_message>
<xml_diff>
--- a/config/parametros.xlsx
+++ b/config/parametros.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diana.acosta\Desktop\CURSO PYTHON\EJERCICIO 3\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CB6EBD-BECE-433C-98E0-DDAC0C5185F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828AED78-7720-4750-A582-F4DA41D9F3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{879D70DC-1290-40BB-97D4-36867B0286A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{879D70DC-1290-40BB-97D4-36867B0286A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros" sheetId="1" r:id="rId1"/>
@@ -354,9 +354,6 @@
     <t>numero_documento;fecha_efectiva;centro_costo</t>
   </si>
   <si>
-    <t>numero_documento:fecha_efectiva</t>
-  </si>
-  <si>
     <t>Consultor Junior</t>
   </si>
   <si>
@@ -406,6 +403,9 @@
   </si>
   <si>
     <t>PERF_GEREN_TI</t>
+  </si>
+  <si>
+    <t>numero_documento;fecha_efectiva</t>
   </si>
 </sst>
 </file>
@@ -870,58 +870,58 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{081E6D7E-F53B-4293-A6BC-A9CB3E36C3CA}" name="Table2" displayName="Table2" ref="A1:D17" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{081E6D7E-F53B-4293-A6BC-A9CB3E36C3CA}" name="Table2" displayName="Table2" ref="A1:D17" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A1:D17" xr:uid="{081E6D7E-F53B-4293-A6BC-A9CB3E36C3CA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D17">
     <sortCondition ref="A2:A17"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{77C1F2ED-938D-4E80-8134-07878D13410F}" name="codigo_cargo" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{ED774E57-E0FB-4A98-9704-2E033F18AD15}" name="nombre_cargo" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{B37B14A9-9656-4D38-9C38-7ED0D9AB8B32}" name="nivel" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{2A36CC35-64E5-4A6A-924C-CDE204460ABF}" name="area" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{77C1F2ED-938D-4E80-8134-07878D13410F}" name="codigo_cargo" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{ED774E57-E0FB-4A98-9704-2E033F18AD15}" name="nombre_cargo" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{B37B14A9-9656-4D38-9C38-7ED0D9AB8B32}" name="nivel" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{2A36CC35-64E5-4A6A-924C-CDE204460ABF}" name="area" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{02A01A09-A269-4B92-98FC-F00FC354A953}" name="Table3" displayName="Table3" ref="A1:C15" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{02A01A09-A269-4B92-98FC-F00FC354A953}" name="Table3" displayName="Table3" ref="A1:C15" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:C15" xr:uid="{02A01A09-A269-4B92-98FC-F00FC354A953}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C15">
     <sortCondition ref="C2:C15"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FEAD6DA2-026C-43FD-AAC9-1E8A167E7682}" name="codigo" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{A8CD677E-49A4-4CE8-8EF4-9585FE76D560}" name="nombre" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{C02FB306-6E65-4270-A3A5-11E6501D7C11}" name="area" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{FEAD6DA2-026C-43FD-AAC9-1E8A167E7682}" name="codigo" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{A8CD677E-49A4-4CE8-8EF4-9585FE76D560}" name="nombre" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{C02FB306-6E65-4270-A3A5-11E6501D7C11}" name="area" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}" name="Table4" displayName="Table4" ref="A1:D17" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}" name="Table4" displayName="Table4" ref="A1:D17" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A1:D17" xr:uid="{B4B8D927-CA4D-49BF-89B0-CFB5CE518CAD}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D14">
     <sortCondition ref="B2:B14"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{473C91A2-BCF7-4D6F-8BF6-61E64B46CCE0}" name="codigo_cargo" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{69A88768-23BB-486C-A0F0-79610F1F7C44}" name="area" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{68BAB88F-0803-48CA-B1F8-E65F18641620}" name="perfil_sistema" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{A1528DB0-D591-4C7B-A8FB-319135B195EE}" name="requiere_aprobacion" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{473C91A2-BCF7-4D6F-8BF6-61E64B46CCE0}" name="codigo_cargo" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{69A88768-23BB-486C-A0F0-79610F1F7C44}" name="area" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{68BAB88F-0803-48CA-B1F8-E65F18641620}" name="perfil_sistema" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{A1528DB0-D591-4C7B-A8FB-319135B195EE}" name="requiere_aprobacion" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}" name="Table5" displayName="Table5" ref="A1:B5" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}" name="Table5" displayName="Table5" ref="A1:B5" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
   <autoFilter ref="A1:B5" xr:uid="{F16AE747-9208-4999-B8C6-E0A429BCB352}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DFC6A082-5976-4820-A3F4-184DF08ECDEE}" name="tipo_novedad" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{3110F81E-BAA3-466D-B6AE-46186B9CD74D}" name="campos_requeridos" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{DFC6A082-5976-4820-A3F4-184DF08ECDEE}" name="tipo_novedad" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{3110F81E-BAA3-466D-B6AE-46186B9CD74D}" name="campos_requeridos" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1254,13 +1254,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1518,7 +1518,7 @@
         <v>31</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C12" s="1">
         <v>2</v>
@@ -1823,7 +1823,7 @@
         <v>39</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>90</v>
@@ -1868,7 +1868,7 @@
         <v>39</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>91</v>
@@ -1883,7 +1883,7 @@
         <v>44</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>91</v>
@@ -1898,7 +1898,7 @@
         <v>44</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>91</v>
@@ -1913,7 +1913,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>91</v>
@@ -1928,7 +1928,7 @@
         <v>44</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>90</v>
@@ -1943,7 +1943,7 @@
         <v>42</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>90</v>
@@ -1958,7 +1958,7 @@
         <v>42</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>90</v>
@@ -1973,7 +1973,7 @@
         <v>42</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>90</v>
@@ -1988,7 +1988,7 @@
         <v>44</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>90</v>
@@ -2003,7 +2003,7 @@
         <v>44</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>90</v>
@@ -2018,7 +2018,7 @@
         <v>44</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>91</v>
@@ -2048,7 +2048,7 @@
         <v>44</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>91</v>
@@ -2109,7 +2109,7 @@
         <v>99</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2297,20 +2297,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="66a9638b-dd80-4936-9407-2514d3c973e6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="66a9638b-dd80-4936-9407-2514d3c973e6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2332,6 +2332,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44E69664-3D00-4936-861C-A6F515DC2017}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA2AE3EE-F1E3-4335-849F-CA480FA8E060}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -2345,12 +2353,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44E69664-3D00-4936-861C-A6F515DC2017}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>